<commit_message>
Finalize YouTube analytics portfolio project
</commit_message>
<xml_diff>
--- a/data/processed/lannkz_youtube_analysis.xlsx
+++ b/data/processed/lannkz_youtube_analysis.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/423d87e852705282/Documents/lannkz-youtube-analysis/data/processed/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="328" documentId="8_{F13BEC6C-2B83-4472-8FBA-B427EE466725}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1BD0E1C8-F477-4C38-9648-F415423FC548}"/>
+  <xr:revisionPtr revIDLastSave="341" documentId="8_{F13BEC6C-2B83-4472-8FBA-B427EE466725}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BF048754-0FEE-4B73-AB54-C53594832F81}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-195" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{B9270838-A669-457C-92D8-1791C4D3D347}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{B9270838-A669-457C-92D8-1791C4D3D347}"/>
   </bookViews>
   <sheets>
     <sheet name="raw_import" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="9" r:id="rId4"/>
+    <pivotCache cacheId="0" r:id="rId4"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -168,9 +168,6 @@
     <t>Blue Lock Only Has 1 Real Coach</t>
   </si>
   <si>
-    <t xml:space="preserve"> -DIPHvPGTnY</t>
-  </si>
-  <si>
     <t>How Scouts Would See LORENZO | Realistic Analysis</t>
   </si>
   <si>
@@ -564,7 +561,10 @@
     <t>avd_duration_ratio</t>
   </si>
   <si>
-    <t>rentention_difference</t>
+    <t>retention_difference</t>
+  </si>
+  <si>
+    <t>-DIPHvPGTnY</t>
   </si>
 </sst>
 </file>
@@ -573,9 +573,9 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
-    <numFmt numFmtId="169" formatCode="0.0000"/>
+    <numFmt numFmtId="165" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -618,9 +618,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -637,18 +637,6 @@
       </fill>
     </dxf>
     <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="169" formatCode="0.0000"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="31" formatCode="[h]:mm:ss"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="yyyy/mm/dd"/>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
     </dxf>
     <dxf>
@@ -659,6 +647,18 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="0.0000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="31" formatCode="[h]:mm:ss"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="yyyy/mm/dd"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1804,7 +1804,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{03B80AC1-9C90-44A1-ADEF-9FC19410A395}" name="PivotTable1" cacheId="9" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{03B80AC1-9C90-44A1-ADEF-9FC19410A395}" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="D1:E5" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="16">
     <pivotField dataField="1" showAll="0"/>
@@ -1908,12 +1908,12 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{39E0E29A-95D6-4669-91C8-FDD00109D317}" name="Table_data" displayName="Table_data" ref="A1:M59" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:M59" xr:uid="{39E0E29A-95D6-4669-91C8-FDD00109D317}"/>
   <tableColumns count="13">
-    <tableColumn id="1" xr3:uid="{053BE77E-9F61-4BDD-AE82-72157BFF0E1B}" uniqueName="1" name="Content" queryTableFieldId="1" dataDxfId="8"/>
-    <tableColumn id="2" xr3:uid="{E420D802-92D9-4375-863E-47FDF0530960}" uniqueName="2" name="Video title" queryTableFieldId="2" dataDxfId="7"/>
-    <tableColumn id="3" xr3:uid="{A83652AC-DC60-4558-894C-EB94C039D093}" uniqueName="3" name="Video publish time" queryTableFieldId="3" dataDxfId="6"/>
+    <tableColumn id="1" xr3:uid="{053BE77E-9F61-4BDD-AE82-72157BFF0E1B}" uniqueName="1" name="Content" queryTableFieldId="1" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{E420D802-92D9-4375-863E-47FDF0530960}" uniqueName="2" name="Video title" queryTableFieldId="2" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{A83652AC-DC60-4558-894C-EB94C039D093}" uniqueName="3" name="Video publish time" queryTableFieldId="3" dataDxfId="2"/>
     <tableColumn id="4" xr3:uid="{925D61CE-F5DA-4F35-81C6-8C5EB1DD75B5}" uniqueName="4" name="video_duration_seconds" queryTableFieldId="4"/>
     <tableColumn id="5" xr3:uid="{F5B0C5C6-E2D1-4C18-A2BA-B679E2795D48}" uniqueName="5" name="Engaged views" queryTableFieldId="5"/>
-    <tableColumn id="6" xr3:uid="{43B616D9-7676-485C-B05F-348AAB79053C}" uniqueName="6" name="Average view duration" queryTableFieldId="6" dataDxfId="5"/>
+    <tableColumn id="6" xr3:uid="{43B616D9-7676-485C-B05F-348AAB79053C}" uniqueName="6" name="Average view duration" queryTableFieldId="6" dataDxfId="1"/>
     <tableColumn id="7" xr3:uid="{5052CDC5-4CF6-41E4-BDA7-FD351F59D40A}" uniqueName="7" name="Average percentage viewed (%)" queryTableFieldId="7"/>
     <tableColumn id="8" xr3:uid="{3583FED4-8600-493C-B2BF-E2167B57E5CB}" uniqueName="8" name="Views" queryTableFieldId="8"/>
     <tableColumn id="9" xr3:uid="{5A0C63CD-2965-4351-BDD0-7CFAF7226846}" uniqueName="9" name="Watch time (hours)" queryTableFieldId="9"/>
@@ -1935,10 +1935,10 @@
   <tableColumns count="18">
     <tableColumn id="1" xr3:uid="{E4A1C0E9-3A23-4885-B939-D634699E83CD}" name="video_id"/>
     <tableColumn id="2" xr3:uid="{F74897C2-E2EB-42E1-AE8F-1A6E0C310F7E}" name="video_title"/>
-    <tableColumn id="3" xr3:uid="{3746B118-2089-4EF4-82C5-776228181DB0}" name="publish_date" dataDxfId="4"/>
+    <tableColumn id="3" xr3:uid="{3746B118-2089-4EF4-82C5-776228181DB0}" name="publish_date" dataDxfId="8"/>
     <tableColumn id="4" xr3:uid="{5F39146F-494D-4375-A6C2-F286D72A8BEB}" name="video_duration_seconds"/>
     <tableColumn id="5" xr3:uid="{ACE6A93E-95EC-463E-AC2D-7B60556668AE}" name="engaged_views"/>
-    <tableColumn id="6" xr3:uid="{B19B2552-F03A-46E5-AEE6-765AF7F860EE}" name="avg_view_duration" dataDxfId="3"/>
+    <tableColumn id="6" xr3:uid="{B19B2552-F03A-46E5-AEE6-765AF7F860EE}" name="avg_view_duration" dataDxfId="7"/>
     <tableColumn id="7" xr3:uid="{980B237C-5B5D-41F4-86BE-E3FBFE6EB3AC}" name="avg_percentage_viewed"/>
     <tableColumn id="8" xr3:uid="{05F399AE-4F03-4377-BCA8-6C44FB8BCC0D}" name="views"/>
     <tableColumn id="9" xr3:uid="{6A9413AB-A7F6-45A6-9013-CAD3CD11F61C}" name="watch_time_hours"/>
@@ -1949,10 +1949,10 @@
     <tableColumn id="14" xr3:uid="{8DCEB431-F004-4A65-B757-5798F3907349}" name="content_type"/>
     <tableColumn id="15" xr3:uid="{FD849346-002E-490F-B3F9-0C3F09B39346}" name="football_relevance"/>
     <tableColumn id="16" xr3:uid="{02B8D4B7-FEDD-441E-9DE7-427DD1E01E43}" name="release_relevance"/>
-    <tableColumn id="17" xr3:uid="{18BB8590-7E3B-449A-9A36-863ED988DAB3}" name="avd_duration_ratio" dataDxfId="2">
+    <tableColumn id="17" xr3:uid="{18BB8590-7E3B-449A-9A36-863ED988DAB3}" name="avd_duration_ratio" dataDxfId="6">
       <calculatedColumnFormula>IFERROR(M2/D2,"")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="18" xr3:uid="{DDE56653-ADC4-4D3F-B824-14675DE3C6F8}" name="rentention_difference" dataDxfId="1">
+    <tableColumn id="18" xr3:uid="{DDE56653-ADC4-4D3F-B824-14675DE3C6F8}" name="retention_difference" dataDxfId="5">
       <calculatedColumnFormula>ABS(Q2*100-G2)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2278,7 +2278,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AE83BB25-765A-43AF-A6CB-57C1188111CD}">
   <dimension ref="A1:M59"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="15.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="81.140625" bestFit="1" customWidth="1"/>
@@ -2295,7 +2295,7 @@
     <col min="13" max="13" width="14.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2336,7 +2336,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13">
       <c r="A2" t="s">
         <v>13</v>
       </c>
@@ -2377,7 +2377,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13">
       <c r="A3" t="s">
         <v>15</v>
       </c>
@@ -2418,7 +2418,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13">
       <c r="A4" t="s">
         <v>17</v>
       </c>
@@ -2459,7 +2459,7 @@
         <v>303</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13">
       <c r="A5" t="s">
         <v>19</v>
       </c>
@@ -2500,7 +2500,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13">
       <c r="A6" t="s">
         <v>21</v>
       </c>
@@ -2541,7 +2541,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:13">
       <c r="A7" t="s">
         <v>23</v>
       </c>
@@ -2582,7 +2582,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:13">
       <c r="A8" t="s">
         <v>25</v>
       </c>
@@ -2623,7 +2623,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:13">
       <c r="A9" t="s">
         <v>27</v>
       </c>
@@ -2664,7 +2664,7 @@
         <v>320</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:13">
       <c r="A10" t="s">
         <v>29</v>
       </c>
@@ -2705,7 +2705,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:13">
       <c r="A11" t="s">
         <v>31</v>
       </c>
@@ -2746,7 +2746,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:13">
       <c r="A12" t="s">
         <v>33</v>
       </c>
@@ -2787,7 +2787,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:13">
       <c r="A13" t="s">
         <v>35</v>
       </c>
@@ -2828,12 +2828,12 @@
         <v>222</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
+    <row r="14" spans="1:13">
+      <c r="A14" s="8" t="s">
+        <v>169</v>
+      </c>
+      <c r="B14" t="s">
         <v>37</v>
-      </c>
-      <c r="B14" t="s">
-        <v>38</v>
       </c>
       <c r="C14" s="1">
         <v>46193</v>
@@ -2869,12 +2869,12 @@
         <v>252</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:13">
       <c r="A15" t="s">
+        <v>38</v>
+      </c>
+      <c r="B15" t="s">
         <v>39</v>
-      </c>
-      <c r="B15" t="s">
-        <v>40</v>
       </c>
       <c r="C15" s="1">
         <v>45774</v>
@@ -2910,12 +2910,12 @@
         <v>406</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:13">
       <c r="A16" t="s">
+        <v>40</v>
+      </c>
+      <c r="B16" t="s">
         <v>41</v>
-      </c>
-      <c r="B16" t="s">
-        <v>42</v>
       </c>
       <c r="C16" s="1">
         <v>46018</v>
@@ -2951,12 +2951,12 @@
         <v>308</v>
       </c>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:13">
       <c r="A17" t="s">
+        <v>42</v>
+      </c>
+      <c r="B17" t="s">
         <v>43</v>
-      </c>
-      <c r="B17" t="s">
-        <v>44</v>
       </c>
       <c r="C17" s="1">
         <v>45962</v>
@@ -2992,12 +2992,12 @@
         <v>335</v>
       </c>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:13">
       <c r="A18" t="s">
+        <v>44</v>
+      </c>
+      <c r="B18" t="s">
         <v>45</v>
-      </c>
-      <c r="B18" t="s">
-        <v>46</v>
       </c>
       <c r="C18" s="1">
         <v>45871</v>
@@ -3033,12 +3033,12 @@
         <v>293</v>
       </c>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:13">
       <c r="A19" t="s">
+        <v>46</v>
+      </c>
+      <c r="B19" t="s">
         <v>47</v>
-      </c>
-      <c r="B19" t="s">
-        <v>48</v>
       </c>
       <c r="C19" s="1">
         <v>46102</v>
@@ -3074,12 +3074,12 @@
         <v>267</v>
       </c>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:13">
       <c r="A20" t="s">
+        <v>48</v>
+      </c>
+      <c r="B20" t="s">
         <v>49</v>
-      </c>
-      <c r="B20" t="s">
-        <v>50</v>
       </c>
       <c r="C20" s="1">
         <v>46200</v>
@@ -3115,12 +3115,12 @@
         <v>171</v>
       </c>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:13">
       <c r="A21" t="s">
+        <v>50</v>
+      </c>
+      <c r="B21" t="s">
         <v>51</v>
-      </c>
-      <c r="B21" t="s">
-        <v>52</v>
       </c>
       <c r="C21" s="1">
         <v>46249</v>
@@ -3156,12 +3156,12 @@
         <v>280</v>
       </c>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:13">
       <c r="A22" t="s">
+        <v>52</v>
+      </c>
+      <c r="B22" t="s">
         <v>53</v>
-      </c>
-      <c r="B22" t="s">
-        <v>54</v>
       </c>
       <c r="C22" s="1">
         <v>46179</v>
@@ -3197,12 +3197,12 @@
         <v>291</v>
       </c>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:13">
       <c r="A23" t="s">
+        <v>54</v>
+      </c>
+      <c r="B23" t="s">
         <v>55</v>
-      </c>
-      <c r="B23" t="s">
-        <v>56</v>
       </c>
       <c r="C23" s="1">
         <v>46151</v>
@@ -3238,12 +3238,12 @@
         <v>274</v>
       </c>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:13">
       <c r="A24" t="s">
+        <v>56</v>
+      </c>
+      <c r="B24" t="s">
         <v>57</v>
-      </c>
-      <c r="B24" t="s">
-        <v>58</v>
       </c>
       <c r="C24" s="1">
         <v>45976</v>
@@ -3279,12 +3279,12 @@
         <v>413</v>
       </c>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:13">
       <c r="A25" t="s">
+        <v>58</v>
+      </c>
+      <c r="B25" t="s">
         <v>59</v>
-      </c>
-      <c r="B25" t="s">
-        <v>60</v>
       </c>
       <c r="C25" s="1">
         <v>46264</v>
@@ -3320,12 +3320,12 @@
         <v>226</v>
       </c>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:13">
       <c r="A26" t="s">
+        <v>60</v>
+      </c>
+      <c r="B26" t="s">
         <v>61</v>
-      </c>
-      <c r="B26" t="s">
-        <v>62</v>
       </c>
       <c r="C26" s="1">
         <v>46039</v>
@@ -3361,12 +3361,12 @@
         <v>351</v>
       </c>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:13">
       <c r="A27" t="s">
+        <v>62</v>
+      </c>
+      <c r="B27" t="s">
         <v>63</v>
-      </c>
-      <c r="B27" t="s">
-        <v>64</v>
       </c>
       <c r="C27" s="1">
         <v>46236</v>
@@ -3402,12 +3402,12 @@
         <v>238</v>
       </c>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:13">
       <c r="A28" t="s">
+        <v>64</v>
+      </c>
+      <c r="B28" t="s">
         <v>65</v>
-      </c>
-      <c r="B28" t="s">
-        <v>66</v>
       </c>
       <c r="C28" s="1">
         <v>45756</v>
@@ -3443,12 +3443,12 @@
         <v>403</v>
       </c>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:13">
       <c r="A29" t="s">
+        <v>66</v>
+      </c>
+      <c r="B29" t="s">
         <v>67</v>
-      </c>
-      <c r="B29" t="s">
-        <v>68</v>
       </c>
       <c r="C29" s="1">
         <v>45801</v>
@@ -3484,12 +3484,12 @@
         <v>221</v>
       </c>
     </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:13">
       <c r="A30" t="s">
+        <v>68</v>
+      </c>
+      <c r="B30" t="s">
         <v>69</v>
-      </c>
-      <c r="B30" t="s">
-        <v>70</v>
       </c>
       <c r="C30" s="1">
         <v>46144</v>
@@ -3525,12 +3525,12 @@
         <v>248</v>
       </c>
     </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:13">
       <c r="A31" t="s">
+        <v>70</v>
+      </c>
+      <c r="B31" t="s">
         <v>71</v>
-      </c>
-      <c r="B31" t="s">
-        <v>72</v>
       </c>
       <c r="C31" s="1">
         <v>45787</v>
@@ -3566,12 +3566,12 @@
         <v>217</v>
       </c>
     </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:13">
       <c r="A32" t="s">
+        <v>72</v>
+      </c>
+      <c r="B32" t="s">
         <v>73</v>
-      </c>
-      <c r="B32" t="s">
-        <v>74</v>
       </c>
       <c r="C32" s="1">
         <v>46207</v>
@@ -3607,12 +3607,12 @@
         <v>267</v>
       </c>
     </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:13">
       <c r="A33" t="s">
+        <v>74</v>
+      </c>
+      <c r="B33" t="s">
         <v>75</v>
-      </c>
-      <c r="B33" t="s">
-        <v>76</v>
       </c>
       <c r="C33" s="1">
         <v>46214</v>
@@ -3648,12 +3648,12 @@
         <v>315</v>
       </c>
     </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:13">
       <c r="A34" t="s">
+        <v>76</v>
+      </c>
+      <c r="B34" t="s">
         <v>77</v>
-      </c>
-      <c r="B34" t="s">
-        <v>78</v>
       </c>
       <c r="C34" s="1">
         <v>46172</v>
@@ -3689,12 +3689,12 @@
         <v>277</v>
       </c>
     </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:13">
       <c r="A35" t="s">
+        <v>78</v>
+      </c>
+      <c r="B35" t="s">
         <v>79</v>
-      </c>
-      <c r="B35" t="s">
-        <v>80</v>
       </c>
       <c r="C35" s="1">
         <v>45948</v>
@@ -3730,12 +3730,12 @@
         <v>251</v>
       </c>
     </row>
-    <row r="36" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:13">
       <c r="A36" t="s">
+        <v>80</v>
+      </c>
+      <c r="B36" t="s">
         <v>81</v>
-      </c>
-      <c r="B36" t="s">
-        <v>82</v>
       </c>
       <c r="C36" s="1">
         <v>46116</v>
@@ -3771,12 +3771,12 @@
         <v>271</v>
       </c>
     </row>
-    <row r="37" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:13">
       <c r="A37" t="s">
+        <v>82</v>
+      </c>
+      <c r="B37" t="s">
         <v>83</v>
-      </c>
-      <c r="B37" t="s">
-        <v>84</v>
       </c>
       <c r="C37" s="1">
         <v>45990</v>
@@ -3812,12 +3812,12 @@
         <v>242</v>
       </c>
     </row>
-    <row r="38" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:13">
       <c r="A38" t="s">
+        <v>84</v>
+      </c>
+      <c r="B38" t="s">
         <v>85</v>
-      </c>
-      <c r="B38" t="s">
-        <v>86</v>
       </c>
       <c r="C38" s="1">
         <v>46222</v>
@@ -3853,12 +3853,12 @@
         <v>319</v>
       </c>
     </row>
-    <row r="39" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:13">
       <c r="A39" t="s">
+        <v>86</v>
+      </c>
+      <c r="B39" t="s">
         <v>87</v>
-      </c>
-      <c r="B39" t="s">
-        <v>88</v>
       </c>
       <c r="C39" s="1">
         <v>45732</v>
@@ -3894,12 +3894,12 @@
         <v>365</v>
       </c>
     </row>
-    <row r="40" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:13">
       <c r="A40" t="s">
+        <v>88</v>
+      </c>
+      <c r="B40" t="s">
         <v>89</v>
-      </c>
-      <c r="B40" t="s">
-        <v>90</v>
       </c>
       <c r="C40" s="1">
         <v>45794</v>
@@ -3935,12 +3935,12 @@
         <v>221</v>
       </c>
     </row>
-    <row r="41" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:13">
       <c r="A41" t="s">
+        <v>90</v>
+      </c>
+      <c r="B41" t="s">
         <v>91</v>
-      </c>
-      <c r="B41" t="s">
-        <v>92</v>
       </c>
       <c r="C41" s="1">
         <v>46278</v>
@@ -3976,12 +3976,12 @@
         <v>274</v>
       </c>
     </row>
-    <row r="42" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:13">
       <c r="A42" t="s">
+        <v>92</v>
+      </c>
+      <c r="B42" t="s">
         <v>93</v>
-      </c>
-      <c r="B42" t="s">
-        <v>94</v>
       </c>
       <c r="C42" s="1">
         <v>46270</v>
@@ -4017,12 +4017,12 @@
         <v>192</v>
       </c>
     </row>
-    <row r="43" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:13">
       <c r="A43" t="s">
+        <v>94</v>
+      </c>
+      <c r="B43" t="s">
         <v>95</v>
-      </c>
-      <c r="B43" t="s">
-        <v>96</v>
       </c>
       <c r="C43" s="1">
         <v>46158</v>
@@ -4058,12 +4058,12 @@
         <v>341</v>
       </c>
     </row>
-    <row r="44" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:13">
       <c r="A44" t="s">
+        <v>96</v>
+      </c>
+      <c r="B44" t="s">
         <v>97</v>
-      </c>
-      <c r="B44" t="s">
-        <v>98</v>
       </c>
       <c r="C44" s="1">
         <v>45920</v>
@@ -4099,12 +4099,12 @@
         <v>303</v>
       </c>
     </row>
-    <row r="45" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:13">
       <c r="A45" t="s">
+        <v>98</v>
+      </c>
+      <c r="B45" t="s">
         <v>99</v>
-      </c>
-      <c r="B45" t="s">
-        <v>100</v>
       </c>
       <c r="C45" s="1">
         <v>45677</v>
@@ -4140,12 +4140,12 @@
         <v>177</v>
       </c>
     </row>
-    <row r="46" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:13">
       <c r="A46" t="s">
+        <v>100</v>
+      </c>
+      <c r="B46" t="s">
         <v>101</v>
-      </c>
-      <c r="B46" t="s">
-        <v>102</v>
       </c>
       <c r="C46" s="1">
         <v>46053</v>
@@ -4181,12 +4181,12 @@
         <v>255</v>
       </c>
     </row>
-    <row r="47" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:13">
       <c r="A47" t="s">
+        <v>102</v>
+      </c>
+      <c r="B47" t="s">
         <v>103</v>
-      </c>
-      <c r="B47" t="s">
-        <v>104</v>
       </c>
       <c r="C47" s="1">
         <v>45717</v>
@@ -4222,12 +4222,12 @@
         <v>318</v>
       </c>
     </row>
-    <row r="48" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:13">
       <c r="A48" t="s">
+        <v>104</v>
+      </c>
+      <c r="B48" t="s">
         <v>105</v>
-      </c>
-      <c r="B48" t="s">
-        <v>106</v>
       </c>
       <c r="C48" s="1">
         <v>46284</v>
@@ -4263,12 +4263,12 @@
         <v>341</v>
       </c>
     </row>
-    <row r="49" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:13">
       <c r="A49" t="s">
+        <v>106</v>
+      </c>
+      <c r="B49" t="s">
         <v>107</v>
-      </c>
-      <c r="B49" t="s">
-        <v>108</v>
       </c>
       <c r="C49" s="1">
         <v>46292</v>
@@ -4304,12 +4304,12 @@
         <v>311</v>
       </c>
     </row>
-    <row r="50" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:13">
       <c r="A50" t="s">
+        <v>108</v>
+      </c>
+      <c r="B50" t="s">
         <v>109</v>
-      </c>
-      <c r="B50" t="s">
-        <v>110</v>
       </c>
       <c r="C50" s="1">
         <v>45765</v>
@@ -4345,12 +4345,12 @@
         <v>199</v>
       </c>
     </row>
-    <row r="51" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:13">
       <c r="A51" t="s">
+        <v>110</v>
+      </c>
+      <c r="B51" t="s">
         <v>111</v>
-      </c>
-      <c r="B51" t="s">
-        <v>112</v>
       </c>
       <c r="C51" s="1">
         <v>45698</v>
@@ -4386,12 +4386,12 @@
         <v>206</v>
       </c>
     </row>
-    <row r="52" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:13">
       <c r="A52" t="s">
+        <v>112</v>
+      </c>
+      <c r="B52" t="s">
         <v>113</v>
-      </c>
-      <c r="B52" t="s">
-        <v>114</v>
       </c>
       <c r="C52" s="1">
         <v>46025</v>
@@ -4427,12 +4427,12 @@
         <v>214</v>
       </c>
     </row>
-    <row r="53" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:13">
       <c r="A53" t="s">
+        <v>114</v>
+      </c>
+      <c r="B53" t="s">
         <v>115</v>
-      </c>
-      <c r="B53" t="s">
-        <v>116</v>
       </c>
       <c r="C53" s="1">
         <v>45815</v>
@@ -4468,12 +4468,12 @@
         <v>383</v>
       </c>
     </row>
-    <row r="54" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:13">
       <c r="A54" t="s">
+        <v>116</v>
+      </c>
+      <c r="B54" t="s">
         <v>117</v>
-      </c>
-      <c r="B54" t="s">
-        <v>118</v>
       </c>
       <c r="C54" s="1">
         <v>45740</v>
@@ -4509,12 +4509,12 @@
         <v>254</v>
       </c>
     </row>
-    <row r="55" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:13">
       <c r="A55" t="s">
+        <v>118</v>
+      </c>
+      <c r="B55" t="s">
         <v>119</v>
-      </c>
-      <c r="B55" t="s">
-        <v>120</v>
       </c>
       <c r="C55" s="1">
         <v>45857</v>
@@ -4550,12 +4550,12 @@
         <v>335</v>
       </c>
     </row>
-    <row r="56" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:13">
       <c r="A56" t="s">
+        <v>120</v>
+      </c>
+      <c r="B56" t="s">
         <v>121</v>
-      </c>
-      <c r="B56" t="s">
-        <v>122</v>
       </c>
       <c r="C56" s="1">
         <v>46074</v>
@@ -4591,12 +4591,12 @@
         <v>150</v>
       </c>
     </row>
-    <row r="57" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:13">
       <c r="A57" t="s">
+        <v>122</v>
+      </c>
+      <c r="B57" t="s">
         <v>123</v>
-      </c>
-      <c r="B57" t="s">
-        <v>124</v>
       </c>
       <c r="C57" s="1">
         <v>45725</v>
@@ -4632,12 +4632,12 @@
         <v>209</v>
       </c>
     </row>
-    <row r="58" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:13">
       <c r="A58" t="s">
+        <v>124</v>
+      </c>
+      <c r="B58" t="s">
         <v>125</v>
-      </c>
-      <c r="B58" t="s">
-        <v>126</v>
       </c>
       <c r="C58" s="1">
         <v>46088</v>
@@ -4673,12 +4673,12 @@
         <v>156</v>
       </c>
     </row>
-    <row r="59" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:13">
       <c r="A59" t="s">
+        <v>126</v>
+      </c>
+      <c r="B59" t="s">
         <v>127</v>
-      </c>
-      <c r="B59" t="s">
-        <v>128</v>
       </c>
       <c r="C59" s="1">
         <v>45657</v>
@@ -4725,7 +4725,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{963FB6BD-D06E-42F0-A2D3-FAE430EF99E0}">
   <dimension ref="A1:T59"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="10.5703125" customWidth="1"/>
     <col min="2" max="2" width="68.85546875" customWidth="1"/>
@@ -4746,68 +4746,68 @@
     <col min="18" max="18" width="23.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:20">
       <c r="A1" t="s">
+        <v>128</v>
+      </c>
+      <c r="B1" t="s">
         <v>129</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" s="1" t="s">
         <v>130</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>131</v>
       </c>
       <c r="D1" t="s">
         <v>3</v>
       </c>
       <c r="E1" t="s">
+        <v>131</v>
+      </c>
+      <c r="F1" t="s">
         <v>132</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>133</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>134</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>135</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>136</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>137</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>138</v>
-      </c>
-      <c r="L1" t="s">
-        <v>139</v>
       </c>
       <c r="M1" t="s">
         <v>12</v>
       </c>
       <c r="N1" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="O1" t="s">
-        <v>164</v>
-      </c>
-      <c r="P1" s="7" t="s">
-        <v>160</v>
+        <v>163</v>
+      </c>
+      <c r="P1" s="6" t="s">
+        <v>159</v>
       </c>
       <c r="Q1" t="s">
+        <v>167</v>
+      </c>
+      <c r="R1" t="s">
         <v>168</v>
       </c>
-      <c r="R1" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:20">
       <c r="A2" t="s">
+        <v>126</v>
+      </c>
+      <c r="B2" t="s">
         <v>127</v>
-      </c>
-      <c r="B2" t="s">
-        <v>128</v>
       </c>
       <c r="C2" s="1">
         <v>45657</v>
@@ -4843,20 +4843,20 @@
         <v>72</v>
       </c>
       <c r="N2" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="O2" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="P2" t="s">
-        <v>159</v>
-      </c>
-      <c r="Q2" s="8">
-        <f>IFERROR(M2/D2,"")</f>
+        <v>158</v>
+      </c>
+      <c r="Q2" s="7">
+        <f t="shared" ref="Q2:Q33" si="0">IFERROR(M2/D2,"")</f>
         <v>0.39779005524861877</v>
       </c>
       <c r="R2">
-        <f>ABS(Q2*100-G2)</f>
+        <f t="shared" ref="R2:R33" si="1">ABS(Q2*100-G2)</f>
         <v>0.3909944751381218</v>
       </c>
       <c r="T2">
@@ -4864,12 +4864,12 @@
         <v>0.3909944751381218</v>
       </c>
     </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:20">
       <c r="A3" t="s">
+        <v>120</v>
+      </c>
+      <c r="B3" t="s">
         <v>121</v>
-      </c>
-      <c r="B3" t="s">
-        <v>122</v>
       </c>
       <c r="C3" s="1">
         <v>46074</v>
@@ -4905,20 +4905,20 @@
         <v>150</v>
       </c>
       <c r="N3" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="O3" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="P3" t="s">
-        <v>157</v>
-      </c>
-      <c r="Q3" s="8">
-        <f>IFERROR(M3/D3,"")</f>
+        <v>156</v>
+      </c>
+      <c r="Q3" s="7">
+        <f t="shared" si="0"/>
         <v>0.47619047619047616</v>
       </c>
       <c r="R3">
-        <f>ABS(Q3*100-G3)</f>
+        <f t="shared" si="1"/>
         <v>0.31095238095238642</v>
       </c>
       <c r="T3">
@@ -4926,12 +4926,12 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:20">
       <c r="A4" t="s">
+        <v>48</v>
+      </c>
+      <c r="B4" t="s">
         <v>49</v>
-      </c>
-      <c r="B4" t="s">
-        <v>50</v>
       </c>
       <c r="C4" s="1">
         <v>46200</v>
@@ -4967,29 +4967,29 @@
         <v>171</v>
       </c>
       <c r="N4" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="O4" t="s">
+        <v>156</v>
+      </c>
+      <c r="P4" t="s">
         <v>157</v>
       </c>
-      <c r="P4" t="s">
-        <v>158</v>
-      </c>
-      <c r="Q4" s="8">
-        <f>IFERROR(M4/D4,"")</f>
+      <c r="Q4" s="7">
+        <f t="shared" si="0"/>
         <v>0.37665198237885461</v>
       </c>
       <c r="R4">
-        <f>ABS(Q4*100-G4)</f>
+        <f t="shared" si="1"/>
         <v>0.19480176211453681</v>
       </c>
     </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:20">
       <c r="A5" t="s">
+        <v>62</v>
+      </c>
+      <c r="B5" t="s">
         <v>63</v>
-      </c>
-      <c r="B5" t="s">
-        <v>64</v>
       </c>
       <c r="C5" s="1">
         <v>46236</v>
@@ -5025,29 +5025,29 @@
         <v>238</v>
       </c>
       <c r="N5" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="O5" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="P5" t="s">
-        <v>157</v>
-      </c>
-      <c r="Q5" s="8">
-        <f>IFERROR(M5/D5,"")</f>
+        <v>156</v>
+      </c>
+      <c r="Q5" s="7">
+        <f t="shared" si="0"/>
         <v>0.44736842105263158</v>
       </c>
       <c r="R5">
-        <f>ABS(Q5*100-G5)</f>
+        <f t="shared" si="1"/>
         <v>0.17315789473683907</v>
       </c>
     </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:20">
       <c r="A6" t="s">
+        <v>70</v>
+      </c>
+      <c r="B6" t="s">
         <v>71</v>
-      </c>
-      <c r="B6" t="s">
-        <v>72</v>
       </c>
       <c r="C6" s="1">
         <v>45787</v>
@@ -5083,29 +5083,29 @@
         <v>217</v>
       </c>
       <c r="N6" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="O6" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="P6" t="s">
-        <v>159</v>
-      </c>
-      <c r="Q6" s="8">
-        <f>IFERROR(M6/D6,"")</f>
+        <v>158</v>
+      </c>
+      <c r="Q6" s="7">
+        <f t="shared" si="0"/>
         <v>0.41811175337186895</v>
       </c>
       <c r="R6">
-        <f>ABS(Q6*100-G6)</f>
+        <f t="shared" si="1"/>
         <v>0.16882466281310116</v>
       </c>
     </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:20">
       <c r="A7" t="s">
+        <v>92</v>
+      </c>
+      <c r="B7" t="s">
         <v>93</v>
-      </c>
-      <c r="B7" t="s">
-        <v>94</v>
       </c>
       <c r="C7" s="1">
         <v>46270</v>
@@ -5141,29 +5141,29 @@
         <v>192</v>
       </c>
       <c r="N7" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="O7" t="s">
+        <v>156</v>
+      </c>
+      <c r="P7" t="s">
         <v>157</v>
       </c>
-      <c r="P7" t="s">
-        <v>158</v>
-      </c>
-      <c r="Q7" s="8">
-        <f>IFERROR(M7/D7,"")</f>
+      <c r="Q7" s="7">
+        <f t="shared" si="0"/>
         <v>0.45714285714285713</v>
       </c>
       <c r="R7">
-        <f>ABS(Q7*100-G7)</f>
+        <f t="shared" si="1"/>
         <v>0.16571428571428726</v>
       </c>
     </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:20">
       <c r="A8" t="s">
+        <v>72</v>
+      </c>
+      <c r="B8" t="s">
         <v>73</v>
-      </c>
-      <c r="B8" t="s">
-        <v>74</v>
       </c>
       <c r="C8" s="1">
         <v>46207</v>
@@ -5199,24 +5199,24 @@
         <v>267</v>
       </c>
       <c r="N8" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="O8" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="P8" t="s">
-        <v>157</v>
-      </c>
-      <c r="Q8" s="8">
-        <f>IFERROR(M8/D8,"")</f>
+        <v>156</v>
+      </c>
+      <c r="Q8" s="7">
+        <f t="shared" si="0"/>
         <v>0.46924428822495606</v>
       </c>
       <c r="R8">
-        <f>ABS(Q8*100-G8)</f>
+        <f t="shared" si="1"/>
         <v>0.16557117750439687</v>
       </c>
     </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:20">
       <c r="A9" t="s">
         <v>25</v>
       </c>
@@ -5257,29 +5257,29 @@
         <v>186</v>
       </c>
       <c r="N9" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="O9" t="s">
+        <v>157</v>
+      </c>
+      <c r="P9" t="s">
         <v>158</v>
       </c>
-      <c r="P9" t="s">
-        <v>159</v>
-      </c>
-      <c r="Q9" s="8">
-        <f>IFERROR(M9/D9,"")</f>
+      <c r="Q9" s="7">
+        <f t="shared" si="0"/>
         <v>0.32068965517241377</v>
       </c>
       <c r="R9">
-        <f>ABS(Q9*100-G9)</f>
+        <f t="shared" si="1"/>
         <v>0.1610344827586232</v>
       </c>
     </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:20">
       <c r="A10" t="s">
+        <v>112</v>
+      </c>
+      <c r="B10" t="s">
         <v>113</v>
-      </c>
-      <c r="B10" t="s">
-        <v>114</v>
       </c>
       <c r="C10" s="1">
         <v>46025</v>
@@ -5315,24 +5315,24 @@
         <v>214</v>
       </c>
       <c r="N10" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="O10" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="P10" t="s">
-        <v>157</v>
-      </c>
-      <c r="Q10" s="8">
-        <f>IFERROR(M10/D10,"")</f>
+        <v>156</v>
+      </c>
+      <c r="Q10" s="7">
+        <f t="shared" si="0"/>
         <v>0.49537037037037035</v>
       </c>
       <c r="R10">
-        <f>ABS(Q10*100-G10)</f>
+        <f t="shared" si="1"/>
         <v>0.15296296296295964</v>
       </c>
     </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:20">
       <c r="A11" t="s">
         <v>33</v>
       </c>
@@ -5373,24 +5373,24 @@
         <v>246</v>
       </c>
       <c r="N11" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="O11" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="P11" t="s">
-        <v>157</v>
-      </c>
-      <c r="Q11" s="8">
-        <f>IFERROR(M11/D11,"")</f>
+        <v>156</v>
+      </c>
+      <c r="Q11" s="7">
+        <f t="shared" si="0"/>
         <v>0.42708333333333331</v>
       </c>
       <c r="R11">
-        <f>ABS(Q11*100-G11)</f>
+        <f t="shared" si="1"/>
         <v>0.14166666666667282</v>
       </c>
     </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:20">
       <c r="A12" t="s">
         <v>13</v>
       </c>
@@ -5431,24 +5431,24 @@
         <v>166</v>
       </c>
       <c r="N12" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="O12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="P12" t="s">
-        <v>159</v>
-      </c>
-      <c r="Q12" s="8">
-        <f>IFERROR(M12/D12,"")</f>
+        <v>158</v>
+      </c>
+      <c r="Q12" s="7">
+        <f t="shared" si="0"/>
         <v>0.48823529411764705</v>
       </c>
       <c r="R12">
-        <f>ABS(Q12*100-G12)</f>
+        <f t="shared" si="1"/>
         <v>0.1364705882352979</v>
       </c>
     </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:20">
       <c r="A13" t="s">
         <v>29</v>
       </c>
@@ -5489,29 +5489,29 @@
         <v>230</v>
       </c>
       <c r="N13" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="O13" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="P13" t="s">
-        <v>157</v>
-      </c>
-      <c r="Q13" s="8">
-        <f>IFERROR(M13/D13,"")</f>
+        <v>156</v>
+      </c>
+      <c r="Q13" s="7">
+        <f t="shared" si="0"/>
         <v>0.34848484848484851</v>
       </c>
       <c r="R13">
-        <f>ABS(Q13*100-G13)</f>
+        <f t="shared" si="1"/>
         <v>0.12151515151514758</v>
       </c>
     </row>
-    <row r="14" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:20">
       <c r="A14" t="s">
+        <v>90</v>
+      </c>
+      <c r="B14" t="s">
         <v>91</v>
-      </c>
-      <c r="B14" t="s">
-        <v>92</v>
       </c>
       <c r="C14" s="1">
         <v>46278</v>
@@ -5547,24 +5547,24 @@
         <v>274</v>
       </c>
       <c r="N14" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="O14" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="P14" t="s">
-        <v>157</v>
-      </c>
-      <c r="Q14" s="8">
-        <f>IFERROR(M14/D14,"")</f>
+        <v>156</v>
+      </c>
+      <c r="Q14" s="7">
+        <f t="shared" si="0"/>
         <v>0.50460405156537758</v>
       </c>
       <c r="R14">
-        <f>ABS(Q14*100-G14)</f>
+        <f t="shared" si="1"/>
         <v>0.10959484346224002</v>
       </c>
     </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:20">
       <c r="A15" t="s">
         <v>19</v>
       </c>
@@ -5605,29 +5605,29 @@
         <v>415</v>
       </c>
       <c r="N15" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="O15" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="P15" t="s">
-        <v>159</v>
-      </c>
-      <c r="Q15" s="8">
-        <f>IFERROR(M15/D15,"")</f>
+        <v>158</v>
+      </c>
+      <c r="Q15" s="7">
+        <f t="shared" si="0"/>
         <v>0.37658802177858441</v>
       </c>
       <c r="R15">
-        <f>ABS(Q15*100-G15)</f>
+        <f t="shared" si="1"/>
         <v>0.10880217785844337</v>
       </c>
     </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:20">
       <c r="A16" t="s">
+        <v>102</v>
+      </c>
+      <c r="B16" t="s">
         <v>103</v>
-      </c>
-      <c r="B16" t="s">
-        <v>104</v>
       </c>
       <c r="C16" s="1">
         <v>45717</v>
@@ -5663,29 +5663,29 @@
         <v>318</v>
       </c>
       <c r="N16" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="O16" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="P16" t="s">
-        <v>159</v>
-      </c>
-      <c r="Q16" s="8">
-        <f>IFERROR(M16/D16,"")</f>
+        <v>158</v>
+      </c>
+      <c r="Q16" s="7">
+        <f t="shared" si="0"/>
         <v>0.48181818181818181</v>
       </c>
       <c r="R16">
-        <f>ABS(Q16*100-G16)</f>
+        <f t="shared" si="1"/>
         <v>0.10818181818181927</v>
       </c>
     </row>
-    <row r="17" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:18">
       <c r="A17" t="s">
+        <v>44</v>
+      </c>
+      <c r="B17" t="s">
         <v>45</v>
-      </c>
-      <c r="B17" t="s">
-        <v>46</v>
       </c>
       <c r="C17" s="1">
         <v>45871</v>
@@ -5721,29 +5721,29 @@
         <v>293</v>
       </c>
       <c r="N17" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="O17" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="P17" t="s">
-        <v>159</v>
-      </c>
-      <c r="Q17" s="8">
-        <f>IFERROR(M17/D17,"")</f>
+        <v>158</v>
+      </c>
+      <c r="Q17" s="7">
+        <f t="shared" si="0"/>
         <v>0.39972714870395637</v>
       </c>
       <c r="R17">
-        <f>ABS(Q17*100-G17)</f>
+        <f t="shared" si="1"/>
         <v>0.10728512960436376</v>
       </c>
     </row>
-    <row r="18" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:18">
       <c r="A18" t="s">
+        <v>80</v>
+      </c>
+      <c r="B18" t="s">
         <v>81</v>
-      </c>
-      <c r="B18" t="s">
-        <v>82</v>
       </c>
       <c r="C18" s="1">
         <v>46116</v>
@@ -5779,29 +5779,29 @@
         <v>271</v>
       </c>
       <c r="N18" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="O18" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="P18" t="s">
-        <v>157</v>
-      </c>
-      <c r="Q18" s="8">
-        <f>IFERROR(M18/D18,"")</f>
+        <v>156</v>
+      </c>
+      <c r="Q18" s="7">
+        <f t="shared" si="0"/>
         <v>0.47964601769911502</v>
       </c>
       <c r="R18">
-        <f>ABS(Q18*100-G18)</f>
+        <f t="shared" si="1"/>
         <v>0.1053982300884968</v>
       </c>
     </row>
-    <row r="19" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:18">
       <c r="A19" t="s">
+        <v>96</v>
+      </c>
+      <c r="B19" t="s">
         <v>97</v>
-      </c>
-      <c r="B19" t="s">
-        <v>98</v>
       </c>
       <c r="C19" s="1">
         <v>45920</v>
@@ -5837,24 +5837,24 @@
         <v>303</v>
       </c>
       <c r="N19" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="O19" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="P19" t="s">
-        <v>157</v>
-      </c>
-      <c r="Q19" s="8">
-        <f>IFERROR(M19/D19,"")</f>
+        <v>156</v>
+      </c>
+      <c r="Q19" s="7">
+        <f t="shared" si="0"/>
         <v>0.44955489614243321</v>
       </c>
       <c r="R19">
-        <f>ABS(Q19*100-G19)</f>
+        <f t="shared" si="1"/>
         <v>0.10451038575668292</v>
       </c>
     </row>
-    <row r="20" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:18">
       <c r="A20" t="s">
         <v>23</v>
       </c>
@@ -5895,29 +5895,29 @@
         <v>242</v>
       </c>
       <c r="N20" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="O20" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="P20" t="s">
-        <v>157</v>
-      </c>
-      <c r="Q20" s="8">
-        <f>IFERROR(M20/D20,"")</f>
+        <v>156</v>
+      </c>
+      <c r="Q20" s="7">
+        <f t="shared" si="0"/>
         <v>0.3522561863173217</v>
       </c>
       <c r="R20">
-        <f>ABS(Q20*100-G20)</f>
+        <f t="shared" si="1"/>
         <v>0.10438136826783051</v>
       </c>
     </row>
-    <row r="21" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:18">
       <c r="A21" t="s">
+        <v>76</v>
+      </c>
+      <c r="B21" t="s">
         <v>77</v>
-      </c>
-      <c r="B21" t="s">
-        <v>78</v>
       </c>
       <c r="C21" s="1">
         <v>46172</v>
@@ -5953,29 +5953,29 @@
         <v>277</v>
       </c>
       <c r="N21" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="O21" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="P21" t="s">
-        <v>159</v>
-      </c>
-      <c r="Q21" s="8">
-        <f>IFERROR(M21/D21,"")</f>
+        <v>158</v>
+      </c>
+      <c r="Q21" s="7">
+        <f t="shared" si="0"/>
         <v>0.46166666666666667</v>
       </c>
       <c r="R21">
-        <f>ABS(Q21*100-G21)</f>
+        <f t="shared" si="1"/>
         <v>0.10333333333333883</v>
       </c>
     </row>
-    <row r="22" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:18">
       <c r="A22" t="s">
+        <v>124</v>
+      </c>
+      <c r="B22" t="s">
         <v>125</v>
-      </c>
-      <c r="B22" t="s">
-        <v>126</v>
       </c>
       <c r="C22" s="1">
         <v>46088</v>
@@ -6011,29 +6011,29 @@
         <v>156</v>
       </c>
       <c r="N22" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="O22" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="P22" t="s">
-        <v>157</v>
-      </c>
-      <c r="Q22" s="8">
-        <f>IFERROR(M22/D22,"")</f>
+        <v>156</v>
+      </c>
+      <c r="Q22" s="7">
+        <f t="shared" si="0"/>
         <v>0.52</v>
       </c>
       <c r="R22">
-        <f>ABS(Q22*100-G22)</f>
+        <f t="shared" si="1"/>
         <v>0.10000000000000142</v>
       </c>
     </row>
-    <row r="23" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:18">
       <c r="A23" t="s">
+        <v>110</v>
+      </c>
+      <c r="B23" t="s">
         <v>111</v>
-      </c>
-      <c r="B23" t="s">
-        <v>112</v>
       </c>
       <c r="C23" s="1">
         <v>45698</v>
@@ -6069,24 +6069,24 @@
         <v>206</v>
       </c>
       <c r="N23" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="O23" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="P23" t="s">
-        <v>157</v>
-      </c>
-      <c r="Q23" s="8">
-        <f>IFERROR(M23/D23,"")</f>
+        <v>156</v>
+      </c>
+      <c r="Q23" s="7">
+        <f t="shared" si="0"/>
         <v>0.42650103519668736</v>
       </c>
       <c r="R23">
-        <f>ABS(Q23*100-G23)</f>
+        <f t="shared" si="1"/>
         <v>8.9896480331269402E-2</v>
       </c>
     </row>
-    <row r="24" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:18">
       <c r="A24" t="s">
         <v>15</v>
       </c>
@@ -6127,29 +6127,29 @@
         <v>216</v>
       </c>
       <c r="N24" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="O24" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="P24" t="s">
-        <v>157</v>
-      </c>
-      <c r="Q24" s="8">
-        <f>IFERROR(M24/D24,"")</f>
+        <v>156</v>
+      </c>
+      <c r="Q24" s="7">
+        <f t="shared" si="0"/>
         <v>0.3323076923076923</v>
       </c>
       <c r="R24">
-        <f>ABS(Q24*100-G24)</f>
+        <f t="shared" si="1"/>
         <v>8.9230769230766782E-2</v>
       </c>
     </row>
-    <row r="25" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:18">
       <c r="A25" t="s">
+        <v>50</v>
+      </c>
+      <c r="B25" t="s">
         <v>51</v>
-      </c>
-      <c r="B25" t="s">
-        <v>52</v>
       </c>
       <c r="C25" s="1">
         <v>46249</v>
@@ -6185,29 +6185,29 @@
         <v>280</v>
       </c>
       <c r="N25" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="O25" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="P25" t="s">
-        <v>157</v>
-      </c>
-      <c r="Q25" s="8">
-        <f>IFERROR(M25/D25,"")</f>
+        <v>156</v>
+      </c>
+      <c r="Q25" s="7">
+        <f t="shared" si="0"/>
         <v>0.42042042042042044</v>
       </c>
       <c r="R25">
-        <f>ABS(Q25*100-G25)</f>
+        <f t="shared" si="1"/>
         <v>8.7957957957961241E-2</v>
       </c>
     </row>
-    <row r="26" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:18">
       <c r="A26" t="s">
+        <v>54</v>
+      </c>
+      <c r="B26" t="s">
         <v>55</v>
-      </c>
-      <c r="B26" t="s">
-        <v>56</v>
       </c>
       <c r="C26" s="1">
         <v>46151</v>
@@ -6243,29 +6243,29 @@
         <v>274</v>
       </c>
       <c r="N26" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="O26" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="P26" t="s">
-        <v>158</v>
-      </c>
-      <c r="Q26" s="8">
-        <f>IFERROR(M26/D26,"")</f>
+        <v>157</v>
+      </c>
+      <c r="Q26" s="7">
+        <f t="shared" si="0"/>
         <v>0.46362098138747887</v>
       </c>
       <c r="R26">
-        <f>ABS(Q26*100-G26)</f>
+        <f t="shared" si="1"/>
         <v>8.7901861252113633E-2</v>
       </c>
     </row>
-    <row r="27" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:18">
       <c r="A27" t="s">
+        <v>66</v>
+      </c>
+      <c r="B27" t="s">
         <v>67</v>
-      </c>
-      <c r="B27" t="s">
-        <v>68</v>
       </c>
       <c r="C27" s="1">
         <v>45801</v>
@@ -6301,29 +6301,29 @@
         <v>221</v>
       </c>
       <c r="N27" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="O27" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="P27" t="s">
-        <v>157</v>
-      </c>
-      <c r="Q27" s="8">
-        <f>IFERROR(M27/D27,"")</f>
+        <v>156</v>
+      </c>
+      <c r="Q27" s="7">
+        <f t="shared" si="0"/>
         <v>0.51276102088167053</v>
       </c>
       <c r="R27">
-        <f>ABS(Q27*100-G27)</f>
+        <f t="shared" si="1"/>
         <v>8.3897911832949035E-2</v>
       </c>
     </row>
-    <row r="28" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:18">
       <c r="A28" t="s">
+        <v>86</v>
+      </c>
+      <c r="B28" t="s">
         <v>87</v>
-      </c>
-      <c r="B28" t="s">
-        <v>88</v>
       </c>
       <c r="C28" s="1">
         <v>45732</v>
@@ -6359,29 +6359,29 @@
         <v>365</v>
       </c>
       <c r="N28" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="O28" t="s">
+        <v>156</v>
+      </c>
+      <c r="P28" t="s">
         <v>157</v>
       </c>
-      <c r="P28" t="s">
-        <v>158</v>
-      </c>
-      <c r="Q28" s="8">
-        <f>IFERROR(M28/D28,"")</f>
+      <c r="Q28" s="7">
+        <f t="shared" si="0"/>
         <v>0.38624338624338622</v>
       </c>
       <c r="R28">
-        <f>ABS(Q28*100-G28)</f>
+        <f t="shared" si="1"/>
         <v>7.566137566138309E-2</v>
       </c>
     </row>
-    <row r="29" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:18">
       <c r="A29" t="s">
+        <v>82</v>
+      </c>
+      <c r="B29" t="s">
         <v>83</v>
-      </c>
-      <c r="B29" t="s">
-        <v>84</v>
       </c>
       <c r="C29" s="1">
         <v>45990</v>
@@ -6417,24 +6417,24 @@
         <v>242</v>
       </c>
       <c r="N29" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="O29" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="P29" t="s">
-        <v>157</v>
-      </c>
-      <c r="Q29" s="8">
-        <f>IFERROR(M29/D29,"")</f>
+        <v>156</v>
+      </c>
+      <c r="Q29" s="7">
+        <f t="shared" si="0"/>
         <v>0.47358121330724068</v>
       </c>
       <c r="R29">
-        <f>ABS(Q29*100-G29)</f>
+        <f t="shared" si="1"/>
         <v>7.1878669275932339E-2</v>
       </c>
     </row>
-    <row r="30" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:18">
       <c r="A30" t="s">
         <v>35</v>
       </c>
@@ -6475,29 +6475,29 @@
         <v>222</v>
       </c>
       <c r="N30" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="O30" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="P30" t="s">
-        <v>158</v>
-      </c>
-      <c r="Q30" s="8">
-        <f>IFERROR(M30/D30,"")</f>
+        <v>157</v>
+      </c>
+      <c r="Q30" s="7">
+        <f t="shared" si="0"/>
         <v>0.38209982788296043</v>
       </c>
       <c r="R30">
-        <f>ABS(Q30*100-G30)</f>
+        <f t="shared" si="1"/>
         <v>7.0017211703955695E-2</v>
       </c>
     </row>
-    <row r="31" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:18">
       <c r="A31" t="s">
+        <v>108</v>
+      </c>
+      <c r="B31" t="s">
         <v>109</v>
-      </c>
-      <c r="B31" t="s">
-        <v>110</v>
       </c>
       <c r="C31" s="1">
         <v>45765</v>
@@ -6533,29 +6533,29 @@
         <v>199</v>
       </c>
       <c r="N31" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="O31" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="P31" t="s">
-        <v>157</v>
-      </c>
-      <c r="Q31" s="8">
-        <f>IFERROR(M31/D31,"")</f>
+        <v>156</v>
+      </c>
+      <c r="Q31" s="7">
+        <f t="shared" si="0"/>
         <v>0.33111480865224624</v>
       </c>
       <c r="R31">
-        <f>ABS(Q31*100-G31)</f>
+        <f t="shared" si="1"/>
         <v>6.8519134775378632E-2</v>
       </c>
     </row>
-    <row r="32" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:18">
       <c r="A32" t="s">
+        <v>58</v>
+      </c>
+      <c r="B32" t="s">
         <v>59</v>
-      </c>
-      <c r="B32" t="s">
-        <v>60</v>
       </c>
       <c r="C32" s="1">
         <v>46264</v>
@@ -6591,29 +6591,29 @@
         <v>226</v>
       </c>
       <c r="N32" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="O32" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="P32" t="s">
-        <v>157</v>
-      </c>
-      <c r="Q32" s="8">
-        <f>IFERROR(M32/D32,"")</f>
+        <v>156</v>
+      </c>
+      <c r="Q32" s="7">
+        <f t="shared" si="0"/>
         <v>0.44752475247524753</v>
       </c>
       <c r="R32">
-        <f>ABS(Q32*100-G32)</f>
+        <f t="shared" si="1"/>
         <v>6.7524752475243588E-2</v>
       </c>
     </row>
-    <row r="33" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:18">
       <c r="A33" t="s">
+        <v>78</v>
+      </c>
+      <c r="B33" t="s">
         <v>79</v>
-      </c>
-      <c r="B33" t="s">
-        <v>80</v>
       </c>
       <c r="C33" s="1">
         <v>45948</v>
@@ -6649,29 +6649,29 @@
         <v>251</v>
       </c>
       <c r="N33" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="O33" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="P33" t="s">
-        <v>157</v>
-      </c>
-      <c r="Q33" s="8">
-        <f>IFERROR(M33/D33,"")</f>
+        <v>156</v>
+      </c>
+      <c r="Q33" s="7">
+        <f t="shared" si="0"/>
         <v>0.47003745318352058</v>
       </c>
       <c r="R33">
-        <f>ABS(Q33*100-G33)</f>
+        <f t="shared" si="1"/>
         <v>6.6254681647940572E-2</v>
       </c>
     </row>
-    <row r="34" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:18">
       <c r="A34" t="s">
+        <v>88</v>
+      </c>
+      <c r="B34" t="s">
         <v>89</v>
-      </c>
-      <c r="B34" t="s">
-        <v>90</v>
       </c>
       <c r="C34" s="1">
         <v>45794</v>
@@ -6707,29 +6707,29 @@
         <v>221</v>
       </c>
       <c r="N34" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="O34" t="s">
+        <v>157</v>
+      </c>
+      <c r="P34" t="s">
         <v>158</v>
       </c>
-      <c r="P34" t="s">
-        <v>159</v>
-      </c>
-      <c r="Q34" s="8">
-        <f>IFERROR(M34/D34,"")</f>
+      <c r="Q34" s="7">
+        <f t="shared" ref="Q34:Q59" si="2">IFERROR(M34/D34,"")</f>
         <v>0.43675889328063239</v>
       </c>
       <c r="R34">
-        <f>ABS(Q34*100-G34)</f>
+        <f t="shared" ref="R34:R65" si="3">ABS(Q34*100-G34)</f>
         <v>6.41106719367599E-2</v>
       </c>
     </row>
-    <row r="35" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:18">
       <c r="A35" t="s">
+        <v>116</v>
+      </c>
+      <c r="B35" t="s">
         <v>117</v>
-      </c>
-      <c r="B35" t="s">
-        <v>118</v>
       </c>
       <c r="C35" s="1">
         <v>45740</v>
@@ -6765,24 +6765,24 @@
         <v>254</v>
       </c>
       <c r="N35" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="O35" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="P35" t="s">
-        <v>157</v>
-      </c>
-      <c r="Q35" s="8">
-        <f>IFERROR(M35/D35,"")</f>
+        <v>156</v>
+      </c>
+      <c r="Q35" s="7">
+        <f t="shared" si="2"/>
         <v>0.41776315789473684</v>
       </c>
       <c r="R35">
-        <f>ABS(Q35*100-G35)</f>
+        <f t="shared" si="3"/>
         <v>6.3684210526318452E-2</v>
       </c>
     </row>
-    <row r="36" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:18">
       <c r="A36" t="s">
         <v>17</v>
       </c>
@@ -6823,29 +6823,29 @@
         <v>303</v>
       </c>
       <c r="N36" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="O36" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="P36" t="s">
-        <v>157</v>
-      </c>
-      <c r="Q36" s="8">
-        <f>IFERROR(M36/D36,"")</f>
+        <v>156</v>
+      </c>
+      <c r="Q36" s="7">
+        <f t="shared" si="2"/>
         <v>0.1696528555431131</v>
       </c>
       <c r="R36">
-        <f>ABS(Q36*100-G36)</f>
+        <f t="shared" si="3"/>
         <v>5.4714445688688329E-2</v>
       </c>
     </row>
-    <row r="37" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:18">
       <c r="A37" t="s">
+        <v>122</v>
+      </c>
+      <c r="B37" t="s">
         <v>123</v>
-      </c>
-      <c r="B37" t="s">
-        <v>124</v>
       </c>
       <c r="C37" s="1">
         <v>45725</v>
@@ -6881,29 +6881,29 @@
         <v>209</v>
       </c>
       <c r="N37" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="O37" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="P37" t="s">
-        <v>157</v>
-      </c>
-      <c r="Q37" s="8">
-        <f>IFERROR(M37/D37,"")</f>
+        <v>156</v>
+      </c>
+      <c r="Q37" s="7">
+        <f t="shared" si="2"/>
         <v>0.50119904076738608</v>
       </c>
       <c r="R37">
-        <f>ABS(Q37*100-G37)</f>
+        <f t="shared" si="3"/>
         <v>5.0095923261395114E-2</v>
       </c>
     </row>
-    <row r="38" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:18">
       <c r="A38" t="s">
+        <v>104</v>
+      </c>
+      <c r="B38" t="s">
         <v>105</v>
-      </c>
-      <c r="B38" t="s">
-        <v>106</v>
       </c>
       <c r="C38" s="1">
         <v>46284</v>
@@ -6939,24 +6939,24 @@
         <v>341</v>
       </c>
       <c r="N38" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="O38" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="P38" t="s">
-        <v>158</v>
-      </c>
-      <c r="Q38" s="8">
-        <f>IFERROR(M38/D38,"")</f>
+        <v>157</v>
+      </c>
+      <c r="Q38" s="7">
+        <f t="shared" si="2"/>
         <v>0.469050894085282</v>
       </c>
       <c r="R38">
-        <f>ABS(Q38*100-G38)</f>
+        <f t="shared" si="3"/>
         <v>4.4910591471804651E-2</v>
       </c>
     </row>
-    <row r="39" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:18">
       <c r="A39" t="s">
         <v>21</v>
       </c>
@@ -6997,29 +6997,29 @@
         <v>264</v>
       </c>
       <c r="N39" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="O39" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="P39" t="s">
-        <v>157</v>
-      </c>
-      <c r="Q39" s="8">
-        <f>IFERROR(M39/D39,"")</f>
+        <v>156</v>
+      </c>
+      <c r="Q39" s="7">
+        <f t="shared" si="2"/>
         <v>0.38995568685376664</v>
       </c>
       <c r="R39">
-        <f>ABS(Q39*100-G39)</f>
+        <f t="shared" si="3"/>
         <v>4.443131462333838E-2</v>
       </c>
     </row>
-    <row r="40" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:18">
       <c r="A40" t="s">
+        <v>56</v>
+      </c>
+      <c r="B40" t="s">
         <v>57</v>
-      </c>
-      <c r="B40" t="s">
-        <v>58</v>
       </c>
       <c r="C40" s="1">
         <v>45976</v>
@@ -7055,29 +7055,29 @@
         <v>413</v>
       </c>
       <c r="N40" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="O40" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="P40" t="s">
-        <v>159</v>
-      </c>
-      <c r="Q40" s="8">
-        <f>IFERROR(M40/D40,"")</f>
+        <v>158</v>
+      </c>
+      <c r="Q40" s="7">
+        <f t="shared" si="2"/>
         <v>0.37106918238993708</v>
       </c>
       <c r="R40">
-        <f>ABS(Q40*100-G40)</f>
+        <f t="shared" si="3"/>
         <v>4.3081761006291686E-2</v>
       </c>
     </row>
-    <row r="41" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:18">
       <c r="A41" t="s">
+        <v>74</v>
+      </c>
+      <c r="B41" t="s">
         <v>75</v>
-      </c>
-      <c r="B41" t="s">
-        <v>76</v>
       </c>
       <c r="C41" s="1">
         <v>46214</v>
@@ -7113,29 +7113,29 @@
         <v>315</v>
       </c>
       <c r="N41" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="O41" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="P41" t="s">
-        <v>157</v>
-      </c>
-      <c r="Q41" s="8">
-        <f>IFERROR(M41/D41,"")</f>
+        <v>156</v>
+      </c>
+      <c r="Q41" s="7">
+        <f t="shared" si="2"/>
         <v>0.44680851063829785</v>
       </c>
       <c r="R41">
-        <f>ABS(Q41*100-G41)</f>
+        <f t="shared" si="3"/>
         <v>3.9148936170214199E-2</v>
       </c>
     </row>
-    <row r="42" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:18">
       <c r="A42" t="s">
+        <v>100</v>
+      </c>
+      <c r="B42" t="s">
         <v>101</v>
-      </c>
-      <c r="B42" t="s">
-        <v>102</v>
       </c>
       <c r="C42" s="1">
         <v>46053</v>
@@ -7171,29 +7171,29 @@
         <v>255</v>
       </c>
       <c r="N42" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="O42" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="P42" t="s">
-        <v>157</v>
-      </c>
-      <c r="Q42" s="8">
-        <f>IFERROR(M42/D42,"")</f>
+        <v>156</v>
+      </c>
+      <c r="Q42" s="7">
+        <f t="shared" si="2"/>
         <v>0.46875</v>
       </c>
       <c r="R42">
-        <f>ABS(Q42*100-G42)</f>
+        <f t="shared" si="3"/>
         <v>3.4999999999996589E-2</v>
       </c>
     </row>
-    <row r="43" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:18">
       <c r="A43" t="s">
+        <v>94</v>
+      </c>
+      <c r="B43" t="s">
         <v>95</v>
-      </c>
-      <c r="B43" t="s">
-        <v>96</v>
       </c>
       <c r="C43" s="1">
         <v>46158</v>
@@ -7229,29 +7229,29 @@
         <v>341</v>
       </c>
       <c r="N43" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="O43" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="P43" t="s">
-        <v>157</v>
-      </c>
-      <c r="Q43" s="8">
-        <f>IFERROR(M43/D43,"")</f>
+        <v>156</v>
+      </c>
+      <c r="Q43" s="7">
+        <f t="shared" si="2"/>
         <v>0.45956873315363883</v>
       </c>
       <c r="R43">
-        <f>ABS(Q43*100-G43)</f>
+        <f t="shared" si="3"/>
         <v>3.3126684636116011E-2</v>
       </c>
     </row>
-    <row r="44" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:18">
       <c r="A44" t="s">
+        <v>42</v>
+      </c>
+      <c r="B44" t="s">
         <v>43</v>
-      </c>
-      <c r="B44" t="s">
-        <v>44</v>
       </c>
       <c r="C44" s="1">
         <v>45962</v>
@@ -7287,29 +7287,29 @@
         <v>335</v>
       </c>
       <c r="N44" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="O44" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="P44" t="s">
-        <v>157</v>
-      </c>
-      <c r="Q44" s="8">
-        <f>IFERROR(M44/D44,"")</f>
+        <v>156</v>
+      </c>
+      <c r="Q44" s="7">
+        <f t="shared" si="2"/>
         <v>0.42458808618504434</v>
       </c>
       <c r="R44">
-        <f>ABS(Q44*100-G44)</f>
+        <f t="shared" si="3"/>
         <v>3.1191381495567327E-2</v>
       </c>
     </row>
-    <row r="45" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:18">
       <c r="A45" t="s">
+        <v>46</v>
+      </c>
+      <c r="B45" t="s">
         <v>47</v>
-      </c>
-      <c r="B45" t="s">
-        <v>48</v>
       </c>
       <c r="C45" s="1">
         <v>46102</v>
@@ -7345,29 +7345,29 @@
         <v>267</v>
       </c>
       <c r="N45" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="O45" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="P45" t="s">
-        <v>157</v>
-      </c>
-      <c r="Q45" s="8">
-        <f>IFERROR(M45/D45,"")</f>
+        <v>156</v>
+      </c>
+      <c r="Q45" s="7">
+        <f t="shared" si="2"/>
         <v>0.4571917808219178</v>
       </c>
       <c r="R45">
-        <f>ABS(Q45*100-G45)</f>
+        <f t="shared" si="3"/>
         <v>3.0821917808218302E-2</v>
       </c>
     </row>
-    <row r="46" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:18">
       <c r="A46" t="s">
+        <v>64</v>
+      </c>
+      <c r="B46" t="s">
         <v>65</v>
-      </c>
-      <c r="B46" t="s">
-        <v>66</v>
       </c>
       <c r="C46" s="1">
         <v>45756</v>
@@ -7403,29 +7403,29 @@
         <v>403</v>
       </c>
       <c r="N46" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="O46" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="P46" t="s">
-        <v>157</v>
-      </c>
-      <c r="Q46" s="8">
-        <f>IFERROR(M46/D46,"")</f>
+        <v>156</v>
+      </c>
+      <c r="Q46" s="7">
+        <f t="shared" si="2"/>
         <v>0.3030075187969925</v>
       </c>
       <c r="R46">
-        <f>ABS(Q46*100-G46)</f>
+        <f t="shared" si="3"/>
         <v>2.9248120300749747E-2</v>
       </c>
     </row>
-    <row r="47" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:18">
       <c r="A47" t="s">
+        <v>68</v>
+      </c>
+      <c r="B47" t="s">
         <v>69</v>
-      </c>
-      <c r="B47" t="s">
-        <v>70</v>
       </c>
       <c r="C47" s="1">
         <v>46144</v>
@@ -7461,29 +7461,29 @@
         <v>248</v>
       </c>
       <c r="N47" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="O47" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="P47" t="s">
-        <v>157</v>
-      </c>
-      <c r="Q47" s="8">
-        <f>IFERROR(M47/D47,"")</f>
+        <v>156</v>
+      </c>
+      <c r="Q47" s="7">
+        <f t="shared" si="2"/>
         <v>0.48062015503875971</v>
       </c>
       <c r="R47">
-        <f>ABS(Q47*100-G47)</f>
+        <f t="shared" si="3"/>
         <v>2.7984496124034308E-2</v>
       </c>
     </row>
-    <row r="48" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:18">
       <c r="A48" t="s">
+        <v>40</v>
+      </c>
+      <c r="B48" t="s">
         <v>41</v>
-      </c>
-      <c r="B48" t="s">
-        <v>42</v>
       </c>
       <c r="C48" s="1">
         <v>46018</v>
@@ -7519,24 +7519,24 @@
         <v>308</v>
       </c>
       <c r="N48" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="O48" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="P48" t="s">
-        <v>157</v>
-      </c>
-      <c r="Q48" s="8">
-        <f>IFERROR(M48/D48,"")</f>
+        <v>156</v>
+      </c>
+      <c r="Q48" s="7">
+        <f t="shared" si="2"/>
         <v>0.42134062927496579</v>
       </c>
       <c r="R48">
-        <f>ABS(Q48*100-G48)</f>
+        <f t="shared" si="3"/>
         <v>2.5937072503417369E-2</v>
       </c>
     </row>
-    <row r="49" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:18">
       <c r="A49" t="s">
         <v>27</v>
       </c>
@@ -7577,29 +7577,29 @@
         <v>320</v>
       </c>
       <c r="N49" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="O49" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="P49" t="s">
-        <v>157</v>
-      </c>
-      <c r="Q49" s="8">
-        <f>IFERROR(M49/D49,"")</f>
+        <v>156</v>
+      </c>
+      <c r="Q49" s="7">
+        <f t="shared" si="2"/>
         <v>0.38834951456310679</v>
       </c>
       <c r="R49">
-        <f>ABS(Q49*100-G49)</f>
+        <f t="shared" si="3"/>
         <v>2.5048543689322855E-2</v>
       </c>
     </row>
-    <row r="50" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:18">
       <c r="A50" t="s">
+        <v>60</v>
+      </c>
+      <c r="B50" t="s">
         <v>61</v>
-      </c>
-      <c r="B50" t="s">
-        <v>62</v>
       </c>
       <c r="C50" s="1">
         <v>46039</v>
@@ -7635,29 +7635,29 @@
         <v>351</v>
       </c>
       <c r="N50" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="O50" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="P50" t="s">
-        <v>157</v>
-      </c>
-      <c r="Q50" s="8">
-        <f>IFERROR(M50/D50,"")</f>
+        <v>156</v>
+      </c>
+      <c r="Q50" s="7">
+        <f t="shared" si="2"/>
         <v>0.42086330935251798</v>
       </c>
       <c r="R50">
-        <f>ABS(Q50*100-G50)</f>
+        <f t="shared" si="3"/>
         <v>2.366906474820496E-2</v>
       </c>
     </row>
-    <row r="51" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:18">
       <c r="A51" t="s">
+        <v>106</v>
+      </c>
+      <c r="B51" t="s">
         <v>107</v>
-      </c>
-      <c r="B51" t="s">
-        <v>108</v>
       </c>
       <c r="C51" s="1">
         <v>46292</v>
@@ -7693,29 +7693,29 @@
         <v>311</v>
       </c>
       <c r="N51" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="O51" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="P51" t="s">
-        <v>157</v>
-      </c>
-      <c r="Q51" s="8">
-        <f>IFERROR(M51/D51,"")</f>
+        <v>156</v>
+      </c>
+      <c r="Q51" s="7">
+        <f t="shared" si="2"/>
         <v>0.50816993464052285</v>
       </c>
       <c r="R51">
-        <f>ABS(Q51*100-G51)</f>
+        <f t="shared" si="3"/>
         <v>2.3006535947715179E-2</v>
       </c>
     </row>
-    <row r="52" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:18">
       <c r="A52" t="s">
+        <v>52</v>
+      </c>
+      <c r="B52" t="s">
         <v>53</v>
-      </c>
-      <c r="B52" t="s">
-        <v>54</v>
       </c>
       <c r="C52" s="1">
         <v>46179</v>
@@ -7751,29 +7751,29 @@
         <v>291</v>
       </c>
       <c r="N52" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="O52" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="P52" t="s">
-        <v>157</v>
-      </c>
-      <c r="Q52" s="8">
-        <f>IFERROR(M52/D52,"")</f>
+        <v>156</v>
+      </c>
+      <c r="Q52" s="7">
+        <f t="shared" si="2"/>
         <v>0.43368107302533532</v>
       </c>
       <c r="R52">
-        <f>ABS(Q52*100-G52)</f>
+        <f t="shared" si="3"/>
         <v>2.1892697466469713E-2</v>
       </c>
     </row>
-    <row r="53" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:18">
       <c r="A53" t="s">
+        <v>38</v>
+      </c>
+      <c r="B53" t="s">
         <v>39</v>
-      </c>
-      <c r="B53" t="s">
-        <v>40</v>
       </c>
       <c r="C53" s="1">
         <v>45774</v>
@@ -7809,29 +7809,29 @@
         <v>406</v>
       </c>
       <c r="N53" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="O53" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="P53" t="s">
-        <v>157</v>
-      </c>
-      <c r="Q53" s="8">
-        <f>IFERROR(M53/D53,"")</f>
+        <v>156</v>
+      </c>
+      <c r="Q53" s="7">
+        <f t="shared" si="2"/>
         <v>0.34641638225255972</v>
       </c>
       <c r="R53">
-        <f>ABS(Q53*100-G53)</f>
+        <f t="shared" si="3"/>
         <v>1.8361774744022341E-2</v>
       </c>
     </row>
-    <row r="54" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:18">
       <c r="A54" t="s">
+        <v>114</v>
+      </c>
+      <c r="B54" t="s">
         <v>115</v>
-      </c>
-      <c r="B54" t="s">
-        <v>116</v>
       </c>
       <c r="C54" s="1">
         <v>45815</v>
@@ -7867,29 +7867,29 @@
         <v>383</v>
       </c>
       <c r="N54" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="O54" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="P54" t="s">
-        <v>157</v>
-      </c>
-      <c r="Q54" s="8">
-        <f>IFERROR(M54/D54,"")</f>
+        <v>156</v>
+      </c>
+      <c r="Q54" s="7">
+        <f t="shared" si="2"/>
         <v>0.45111896348645464</v>
       </c>
       <c r="R54">
-        <f>ABS(Q54*100-G54)</f>
+        <f t="shared" si="3"/>
         <v>1.810365135453651E-2</v>
       </c>
     </row>
-    <row r="55" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A55" t="s">
+    <row r="55" spans="1:18">
+      <c r="A55" s="8" t="s">
+        <v>169</v>
+      </c>
+      <c r="B55" t="s">
         <v>37</v>
-      </c>
-      <c r="B55" t="s">
-        <v>38</v>
       </c>
       <c r="C55" s="1">
         <v>46193</v>
@@ -7925,29 +7925,29 @@
         <v>252</v>
       </c>
       <c r="N55" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="O55" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="P55" t="s">
-        <v>157</v>
-      </c>
-      <c r="Q55" s="8">
-        <f>IFERROR(M55/D55,"")</f>
+        <v>156</v>
+      </c>
+      <c r="Q55" s="7">
+        <f t="shared" si="2"/>
         <v>0.40384615384615385</v>
       </c>
       <c r="R55">
-        <f>ABS(Q55*100-G55)</f>
+        <f t="shared" si="3"/>
         <v>1.5384615384611777E-2</v>
       </c>
     </row>
-    <row r="56" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:18">
       <c r="A56" t="s">
+        <v>84</v>
+      </c>
+      <c r="B56" t="s">
         <v>85</v>
-      </c>
-      <c r="B56" t="s">
-        <v>86</v>
       </c>
       <c r="C56" s="1">
         <v>46222</v>
@@ -7983,29 +7983,29 @@
         <v>319</v>
       </c>
       <c r="N56" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="O56" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="P56" t="s">
-        <v>157</v>
-      </c>
-      <c r="Q56" s="8">
-        <f>IFERROR(M56/D56,"")</f>
+        <v>156</v>
+      </c>
+      <c r="Q56" s="7">
+        <f t="shared" si="2"/>
         <v>0.46705710102489018</v>
       </c>
       <c r="R56">
-        <f>ABS(Q56*100-G56)</f>
+        <f t="shared" si="3"/>
         <v>1.4289897510984417E-2</v>
       </c>
     </row>
-    <row r="57" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:18">
       <c r="A57" t="s">
+        <v>118</v>
+      </c>
+      <c r="B57" t="s">
         <v>119</v>
-      </c>
-      <c r="B57" t="s">
-        <v>120</v>
       </c>
       <c r="C57" s="1">
         <v>45857</v>
@@ -8041,24 +8041,24 @@
         <v>335</v>
       </c>
       <c r="N57" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="O57" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="P57" t="s">
-        <v>157</v>
-      </c>
-      <c r="Q57" s="8">
-        <f>IFERROR(M57/D57,"")</f>
+        <v>156</v>
+      </c>
+      <c r="Q57" s="7">
+        <f t="shared" si="2"/>
         <v>0.41256157635467983</v>
       </c>
       <c r="R57">
-        <f>ABS(Q57*100-G57)</f>
+        <f t="shared" si="3"/>
         <v>1.384236453201737E-2</v>
       </c>
     </row>
-    <row r="58" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:18">
       <c r="A58" t="s">
         <v>31</v>
       </c>
@@ -8099,29 +8099,29 @@
         <v>242</v>
       </c>
       <c r="N58" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="O58" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="P58" t="s">
-        <v>159</v>
-      </c>
-      <c r="Q58" s="8">
-        <f>IFERROR(M58/D58,"")</f>
+        <v>158</v>
+      </c>
+      <c r="Q58" s="7">
+        <f t="shared" si="2"/>
         <v>0.38782051282051283</v>
       </c>
       <c r="R58">
-        <f>ABS(Q58*100-G58)</f>
+        <f t="shared" si="3"/>
         <v>7.9487179487145454E-3</v>
       </c>
     </row>
-    <row r="59" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:18">
       <c r="A59" t="s">
+        <v>98</v>
+      </c>
+      <c r="B59" t="s">
         <v>99</v>
-      </c>
-      <c r="B59" t="s">
-        <v>100</v>
       </c>
       <c r="C59" s="1">
         <v>45677</v>
@@ -8157,20 +8157,20 @@
         <v>177</v>
       </c>
       <c r="N59" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="O59" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="P59" t="s">
-        <v>159</v>
-      </c>
-      <c r="Q59" s="8">
-        <f>IFERROR(M59/D59,"")</f>
+        <v>158</v>
+      </c>
+      <c r="Q59" s="7">
+        <f t="shared" si="2"/>
         <v>0.35399999999999998</v>
       </c>
       <c r="R59">
-        <f>ABS(Q59*100-G59)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -8196,7 +8196,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{943A209C-037B-4F2F-87A0-C0C3C2F8EBB7}">
   <dimension ref="A1:E16"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="18.42578125" customWidth="1"/>
     <col min="2" max="2" width="80.42578125" customWidth="1"/>
@@ -8206,146 +8206,146 @@
     <col min="9" max="9" width="11.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5">
       <c r="A1" t="s">
+        <v>139</v>
+      </c>
+      <c r="B1" t="s">
         <v>140</v>
       </c>
-      <c r="B1" t="s">
+      <c r="D1" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="E1" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2" t="s">
         <v>141</v>
       </c>
-      <c r="D1" s="4" t="s">
-        <v>154</v>
-      </c>
-      <c r="E1" t="s">
+      <c r="B2" t="s">
+        <v>146</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>158</v>
+      </c>
+      <c r="E2">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
+      <c r="A3" t="s">
+        <v>142</v>
+      </c>
+      <c r="B3" t="s">
+        <v>147</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>156</v>
+      </c>
+      <c r="E3">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="A4" t="s">
+        <v>145</v>
+      </c>
+      <c r="B4" t="s">
+        <v>148</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>157</v>
+      </c>
+      <c r="E4">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
+      <c r="A5" t="s">
+        <v>143</v>
+      </c>
+      <c r="B5" t="s">
+        <v>149</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="E5">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
+      <c r="A6" t="s">
+        <v>144</v>
+      </c>
+      <c r="B6" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5">
+      <c r="A8" t="s">
         <v>155</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>142</v>
-      </c>
-      <c r="B2" t="s">
-        <v>147</v>
-      </c>
-      <c r="D2" s="5" t="s">
+      <c r="B8" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5">
+      <c r="A9" t="s">
+        <v>156</v>
+      </c>
+      <c r="B9" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5">
+      <c r="A10" t="s">
+        <v>157</v>
+      </c>
+      <c r="B10" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5">
+      <c r="A11" t="s">
+        <v>158</v>
+      </c>
+      <c r="B11" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5">
+      <c r="A13" t="s">
         <v>159</v>
       </c>
-      <c r="E2" s="6">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>143</v>
-      </c>
-      <c r="B3" t="s">
-        <v>148</v>
-      </c>
-      <c r="D3" s="5" t="s">
+      <c r="B13" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5">
+      <c r="A14" t="s">
+        <v>156</v>
+      </c>
+      <c r="B14" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5">
+      <c r="A15" t="s">
         <v>157</v>
       </c>
-      <c r="E3" s="6">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>146</v>
-      </c>
-      <c r="B4" t="s">
-        <v>149</v>
-      </c>
-      <c r="D4" s="5" t="s">
+      <c r="B15" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5">
+      <c r="A16" t="s">
         <v>158</v>
       </c>
-      <c r="E4" s="6">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>144</v>
-      </c>
-      <c r="B5" t="s">
-        <v>150</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>153</v>
-      </c>
-      <c r="E5" s="6">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>145</v>
-      </c>
-      <c r="B6" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>156</v>
-      </c>
-      <c r="B8" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>157</v>
-      </c>
-      <c r="B9" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>158</v>
-      </c>
-      <c r="B10" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>159</v>
-      </c>
-      <c r="B11" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>160</v>
-      </c>
-      <c r="B13" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>157</v>
-      </c>
-      <c r="B14" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>158</v>
-      </c>
-      <c r="B15" t="s">
+      <c r="B16" t="s">
         <v>162</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>159</v>
-      </c>
-      <c r="B16" t="s">
-        <v>163</v>
       </c>
     </row>
   </sheetData>

</xml_diff>